<commit_message>
Frase pública de donación sin cifra, texto literal de Khalid, tarifa real de AW (2,95/4,00/6,50) y desglose de beneficio por producto, logo circular + favicon y correos automáticos al cliente
</commit_message>
<xml_diff>
--- a/docs/GRANKHA_Auditoria_Precios.xlsx
+++ b/docs/GRANKHA_Auditoria_Precios.xlsx
@@ -568,7 +568,7 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>8.15703240539365</v>
+        <v>9.853085036972596</v>
       </c>
     </row>
     <row r="11">
@@ -578,7 +578,7 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>16.90138060026098</v>
+        <v>18.55495954762941</v>
       </c>
     </row>
     <row r="12">
@@ -588,7 +588,7 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>16.41178650137741</v>
+        <v>17.71545316804408</v>
       </c>
     </row>
     <row r="13">
@@ -598,7 +598,7 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>0.2934576067200537</v>
+        <v>0.360422045209625</v>
       </c>
     </row>
     <row r="14">
@@ -839,13 +839,13 @@
         </is>
       </c>
       <c r="L5" s="4" t="n">
-        <v>8.56982438016529</v>
+        <v>10.56982438016529</v>
       </c>
       <c r="M5" s="4" t="n">
-        <v>15.39814876033058</v>
+        <v>17.39814876033058</v>
       </c>
       <c r="N5" s="5" t="n">
-        <v>0.2810159214092141</v>
+        <v>0.3465985772357724</v>
       </c>
       <c r="O5" s="7" t="inlineStr">
         <is>
@@ -903,13 +903,13 @@
         </is>
       </c>
       <c r="L6" s="4" t="n">
-        <v>8.56982438016529</v>
+        <v>10.56982438016529</v>
       </c>
       <c r="M6" s="4" t="n">
-        <v>15.39814876033058</v>
+        <v>17.39814876033058</v>
       </c>
       <c r="N6" s="5" t="n">
-        <v>0.2810159214092141</v>
+        <v>0.3465985772357724</v>
       </c>
       <c r="O6" s="7" t="inlineStr">
         <is>
@@ -967,13 +967,13 @@
         </is>
       </c>
       <c r="L7" s="4" t="n">
-        <v>8.56982438016529</v>
+        <v>10.56982438016529</v>
       </c>
       <c r="M7" s="4" t="n">
-        <v>15.39814876033058</v>
+        <v>17.39814876033058</v>
       </c>
       <c r="N7" s="5" t="n">
-        <v>0.2810159214092141</v>
+        <v>0.3465985772357724</v>
       </c>
       <c r="O7" s="7" t="inlineStr">
         <is>
@@ -1031,13 +1031,13 @@
         </is>
       </c>
       <c r="L8" s="4" t="n">
-        <v>8.56982438016529</v>
+        <v>10.56982438016529</v>
       </c>
       <c r="M8" s="4" t="n">
-        <v>15.39814876033058</v>
+        <v>17.39814876033058</v>
       </c>
       <c r="N8" s="5" t="n">
-        <v>0.2810159214092141</v>
+        <v>0.3465985772357724</v>
       </c>
       <c r="O8" s="7" t="inlineStr">
         <is>
@@ -1095,13 +1095,13 @@
         </is>
       </c>
       <c r="L9" s="4" t="n">
-        <v>8.56982438016529</v>
+        <v>10.56982438016529</v>
       </c>
       <c r="M9" s="4" t="n">
-        <v>15.39814876033058</v>
+        <v>17.39814876033058</v>
       </c>
       <c r="N9" s="5" t="n">
-        <v>0.2810159214092141</v>
+        <v>0.3465985772357724</v>
       </c>
       <c r="O9" s="7" t="inlineStr">
         <is>
@@ -1159,13 +1159,13 @@
         </is>
       </c>
       <c r="L10" s="4" t="n">
-        <v>8.56982438016529</v>
+        <v>10.56982438016529</v>
       </c>
       <c r="M10" s="4" t="n">
-        <v>15.39814876033058</v>
+        <v>17.39814876033058</v>
       </c>
       <c r="N10" s="5" t="n">
-        <v>0.2810159214092141</v>
+        <v>0.3465985772357724</v>
       </c>
       <c r="O10" s="7" t="inlineStr">
         <is>
@@ -1223,13 +1223,13 @@
         </is>
       </c>
       <c r="L11" s="4" t="n">
-        <v>3.316464876033059</v>
+        <v>5.316464876033058</v>
       </c>
       <c r="M11" s="4" t="n">
-        <v>4.891429752066117</v>
+        <v>6.891429752066117</v>
       </c>
       <c r="N11" s="5" t="n">
-        <v>0.1832384703196348</v>
+        <v>0.2937407534246576</v>
       </c>
       <c r="O11" s="7" t="inlineStr">
         <is>
@@ -1287,13 +1287,13 @@
         </is>
       </c>
       <c r="L12" s="4" t="n">
-        <v>3.316464876033059</v>
+        <v>5.316464876033058</v>
       </c>
       <c r="M12" s="4" t="n">
-        <v>4.891429752066117</v>
+        <v>6.891429752066117</v>
       </c>
       <c r="N12" s="5" t="n">
-        <v>0.1832384703196348</v>
+        <v>0.2937407534246576</v>
       </c>
       <c r="O12" s="7" t="inlineStr">
         <is>
@@ -1351,13 +1351,13 @@
         </is>
       </c>
       <c r="L13" s="4" t="n">
-        <v>3.316464876033059</v>
+        <v>5.316464876033058</v>
       </c>
       <c r="M13" s="4" t="n">
-        <v>4.891429752066117</v>
+        <v>6.891429752066117</v>
       </c>
       <c r="N13" s="5" t="n">
-        <v>0.1832384703196348</v>
+        <v>0.2937407534246576</v>
       </c>
       <c r="O13" s="7" t="inlineStr">
         <is>
@@ -1415,13 +1415,13 @@
         </is>
       </c>
       <c r="L14" s="4" t="n">
-        <v>5.914956611570248</v>
+        <v>7.914956611570247</v>
       </c>
       <c r="M14" s="4" t="n">
-        <v>10.0884132231405</v>
+        <v>12.0884132231405</v>
       </c>
       <c r="N14" s="5" t="n">
-        <v>0.2393678093645485</v>
+        <v>0.3203042642140468</v>
       </c>
       <c r="O14" s="7" t="inlineStr">
         <is>
@@ -1479,13 +1479,13 @@
         </is>
       </c>
       <c r="L15" s="4" t="n">
-        <v>5.914956611570248</v>
+        <v>7.914956611570247</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>10.0884132231405</v>
+        <v>12.0884132231405</v>
       </c>
       <c r="N15" s="5" t="n">
-        <v>0.2393678093645485</v>
+        <v>0.3203042642140468</v>
       </c>
       <c r="O15" s="7" t="inlineStr">
         <is>
@@ -1543,13 +1543,13 @@
         </is>
       </c>
       <c r="L16" s="4" t="n">
-        <v>5.914956611570248</v>
+        <v>7.914956611570247</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>10.0884132231405</v>
+        <v>12.0884132231405</v>
       </c>
       <c r="N16" s="5" t="n">
-        <v>0.2393678093645485</v>
+        <v>0.3203042642140468</v>
       </c>
       <c r="O16" s="7" t="inlineStr">
         <is>
@@ -1607,13 +1607,13 @@
         </is>
       </c>
       <c r="L17" s="4" t="n">
-        <v>6.915576446280991</v>
+        <v>8.915576446280991</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>12.08965289256198</v>
+        <v>14.08965289256198</v>
       </c>
       <c r="N17" s="5" t="n">
-        <v>0.2397664040114613</v>
+        <v>0.3091073782234957</v>
       </c>
       <c r="O17" s="7" t="inlineStr">
         <is>
@@ -1671,13 +1671,13 @@
         </is>
       </c>
       <c r="L18" s="4" t="n">
-        <v>6.915576446280991</v>
+        <v>8.915576446280991</v>
       </c>
       <c r="M18" s="4" t="n">
-        <v>12.08965289256198</v>
+        <v>14.08965289256198</v>
       </c>
       <c r="N18" s="5" t="n">
-        <v>0.2397664040114613</v>
+        <v>0.3091073782234957</v>
       </c>
       <c r="O18" s="7" t="inlineStr">
         <is>
@@ -1735,13 +1735,13 @@
         </is>
       </c>
       <c r="L19" s="4" t="n">
-        <v>6.915576446280991</v>
+        <v>8.915576446280991</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>12.08965289256198</v>
+        <v>14.08965289256198</v>
       </c>
       <c r="N19" s="5" t="n">
-        <v>0.2397664040114613</v>
+        <v>0.3091073782234957</v>
       </c>
       <c r="O19" s="7" t="inlineStr">
         <is>
@@ -1799,13 +1799,13 @@
         </is>
       </c>
       <c r="L20" s="4" t="n">
-        <v>6.25047314049587</v>
+        <v>8.250473140495869</v>
       </c>
       <c r="M20" s="4" t="n">
-        <v>6.819446280991738</v>
+        <v>8.819446280991738</v>
       </c>
       <c r="N20" s="5" t="n">
-        <v>0.5441059352517986</v>
+        <v>0.718206654676259</v>
       </c>
       <c r="O20" s="7" t="inlineStr">
         <is>
@@ -1863,13 +1863,13 @@
         </is>
       </c>
       <c r="L21" s="4" t="n">
-        <v>7.848345041322314</v>
+        <v>9.848345041322313</v>
       </c>
       <c r="M21" s="4" t="n">
-        <v>10.01519008264463</v>
+        <v>12.01519008264463</v>
       </c>
       <c r="N21" s="5" t="n">
-        <v>0.5619229289940828</v>
+        <v>0.7051181952662722</v>
       </c>
       <c r="O21" s="7" t="inlineStr">
         <is>
@@ -1927,13 +1927,13 @@
         </is>
       </c>
       <c r="L22" s="4" t="n">
-        <v>8.231084710743801</v>
+        <v>10.2310847107438</v>
       </c>
       <c r="M22" s="4" t="n">
-        <v>14.7206694214876</v>
+        <v>16.7206694214876</v>
       </c>
       <c r="N22" s="5" t="n">
-        <v>0.3702458178438661</v>
+        <v>0.4602086431226766</v>
       </c>
       <c r="O22" s="7" t="inlineStr">
         <is>
@@ -1991,13 +1991,13 @@
         </is>
       </c>
       <c r="L23" s="4" t="n">
-        <v>8.300446280991739</v>
+        <v>10.30044628099174</v>
       </c>
       <c r="M23" s="4" t="n">
-        <v>22.64089256198348</v>
+        <v>24.64089256198348</v>
       </c>
       <c r="N23" s="5" t="n">
-        <v>0.2517177944862156</v>
+        <v>0.3123694235588973</v>
       </c>
       <c r="O23" s="7" t="inlineStr">
         <is>
@@ -2055,13 +2055,13 @@
         </is>
       </c>
       <c r="L24" s="4" t="n">
-        <v>8.588566115702477</v>
+        <v>9.538566115702478</v>
       </c>
       <c r="M24" s="4" t="n">
-        <v>23.17313223140496</v>
+        <v>24.16713223140496</v>
       </c>
       <c r="N24" s="5" t="n">
-        <v>0.2314513363028953</v>
+        <v>0.2570526726057906</v>
       </c>
       <c r="O24" s="7" t="inlineStr">
         <is>
@@ -2119,13 +2119,13 @@
         </is>
       </c>
       <c r="L25" s="4" t="n">
-        <v>10.18995661157025</v>
+        <v>12.18995661157025</v>
       </c>
       <c r="M25" s="4" t="n">
-        <v>18.6384132231405</v>
+        <v>19.5884132231405</v>
       </c>
       <c r="N25" s="5" t="n">
-        <v>0.4123694816053512</v>
+        <v>0.4933059364548494</v>
       </c>
       <c r="O25" s="7" t="inlineStr">
         <is>
@@ -2183,13 +2183,13 @@
         </is>
       </c>
       <c r="L26" s="4" t="n">
-        <v>7.905969008264462</v>
+        <v>9.905969008264462</v>
       </c>
       <c r="M26" s="4" t="n">
-        <v>10.13043801652892</v>
+        <v>12.13043801652892</v>
       </c>
       <c r="N26" s="5" t="n">
-        <v>0.5344258379888268</v>
+        <v>0.6696213687150838</v>
       </c>
       <c r="O26" s="7" t="inlineStr">
         <is>
@@ -2247,13 +2247,13 @@
         </is>
       </c>
       <c r="L27" s="4" t="n">
-        <v>5.314185950413225</v>
+        <v>7.314185950413224</v>
       </c>
       <c r="M27" s="4" t="n">
-        <v>16.66837190082645</v>
+        <v>17.61837190082645</v>
       </c>
       <c r="N27" s="5" t="n">
-        <v>0.1288610220440882</v>
+        <v>0.1773580160320641</v>
       </c>
       <c r="O27" s="7" t="inlineStr">
         <is>
@@ -2311,13 +2311,13 @@
         </is>
       </c>
       <c r="L28" s="4" t="n">
-        <v>12.38109297520661</v>
+        <v>14.38109297520661</v>
       </c>
       <c r="M28" s="4" t="n">
-        <v>19.08068595041322</v>
+        <v>21.08068595041322</v>
       </c>
       <c r="N28" s="5" t="n">
-        <v>0.7926519841269841</v>
+        <v>0.9206943121693121</v>
       </c>
       <c r="O28" s="7" t="inlineStr">
         <is>
@@ -2375,13 +2375,13 @@
         </is>
       </c>
       <c r="L29" s="4" t="n">
-        <v>8.758576446280992</v>
+        <v>10.75857644628099</v>
       </c>
       <c r="M29" s="4" t="n">
-        <v>15.77565289256198</v>
+        <v>16.72565289256199</v>
       </c>
       <c r="N29" s="5" t="n">
-        <v>0.303664111747851</v>
+        <v>0.3730050859598854</v>
       </c>
       <c r="O29" s="7" t="inlineStr">
         <is>
@@ -2439,13 +2439,13 @@
         </is>
       </c>
       <c r="L30" s="4" t="n">
-        <v>8.29406611570248</v>
+        <v>9.244066115702481</v>
       </c>
       <c r="M30" s="4" t="n">
-        <v>22.62813223140496</v>
+        <v>23.57813223140496</v>
       </c>
       <c r="N30" s="5" t="n">
-        <v>0.2235149220489978</v>
+        <v>0.2491162583518931</v>
       </c>
       <c r="O30" s="7" t="inlineStr">
         <is>
@@ -2503,13 +2503,13 @@
         </is>
       </c>
       <c r="L31" s="4" t="n">
-        <v>5.982446280991737</v>
+        <v>6.932446280991737</v>
       </c>
       <c r="M31" s="4" t="n">
-        <v>17.27889256198348</v>
+        <v>18.95489256198347</v>
       </c>
       <c r="N31" s="5" t="n">
-        <v>0.1814225563909775</v>
+        <v>0.2102320802005013</v>
       </c>
       <c r="O31" s="7" t="inlineStr">
         <is>
@@ -2567,13 +2567,13 @@
         </is>
       </c>
       <c r="L32" s="4" t="n">
-        <v>10.76905785123967</v>
+        <v>11.71905785123967</v>
       </c>
       <c r="M32" s="4" t="n">
-        <v>26.25811570247933</v>
+        <v>28.52811570247933</v>
       </c>
       <c r="N32" s="5" t="n">
-        <v>0.2463243856332702</v>
+        <v>0.2680540642722117</v>
       </c>
       <c r="O32" s="7" t="inlineStr">
         <is>
@@ -2631,13 +2631,13 @@
         </is>
       </c>
       <c r="L33" s="4" t="n">
-        <v>11.06894834710744</v>
+        <v>12.01894834710744</v>
       </c>
       <c r="M33" s="4" t="n">
-        <v>20.39639669421488</v>
+        <v>21.34639669421487</v>
       </c>
       <c r="N33" s="5" t="n">
-        <v>0.3533885883905014</v>
+        <v>0.3837184036939315</v>
       </c>
       <c r="O33" s="7" t="inlineStr">
         <is>
@@ -2695,13 +2695,13 @@
         </is>
       </c>
       <c r="L34" s="4" t="n">
-        <v>11.06894834710744</v>
+        <v>12.01894834710744</v>
       </c>
       <c r="M34" s="4" t="n">
-        <v>20.39639669421488</v>
+        <v>21.34639669421487</v>
       </c>
       <c r="N34" s="5" t="n">
-        <v>0.3533885883905014</v>
+        <v>0.3837184036939315</v>
       </c>
       <c r="O34" s="7" t="inlineStr">
         <is>
@@ -2759,13 +2759,13 @@
         </is>
       </c>
       <c r="L35" s="4" t="n">
-        <v>7.876066115702478</v>
+        <v>8.826066115702478</v>
       </c>
       <c r="M35" s="4" t="n">
-        <v>21.24213223140496</v>
+        <v>22.74213223140496</v>
       </c>
       <c r="N35" s="5" t="n">
-        <v>0.2122503340757238</v>
+        <v>0.2378516703786191</v>
       </c>
       <c r="O35" s="7" t="inlineStr">
         <is>
@@ -2823,13 +2823,13 @@
         </is>
       </c>
       <c r="L36" s="4" t="n">
-        <v>11.71205371900826</v>
+        <v>12.66205371900826</v>
       </c>
       <c r="M36" s="4" t="n">
-        <v>28.21010743801652</v>
+        <v>30.41410743801652</v>
       </c>
       <c r="N36" s="5" t="n">
-        <v>0.2490612478031634</v>
+        <v>0.2692633567662565</v>
       </c>
       <c r="O36" s="7" t="inlineStr">
         <is>
@@ -2887,13 +2887,13 @@
         </is>
       </c>
       <c r="L37" s="4" t="n">
-        <v>7.587946280991738</v>
+        <v>9.587946280991737</v>
       </c>
       <c r="M37" s="4" t="n">
-        <v>21.21589256198347</v>
+        <v>22.16589256198348</v>
       </c>
       <c r="N37" s="5" t="n">
-        <v>0.2301106516290727</v>
+        <v>0.2907622807017544</v>
       </c>
       <c r="O37" s="7" t="inlineStr">
         <is>
@@ -2951,13 +2951,13 @@
         </is>
       </c>
       <c r="L38" s="4" t="n">
-        <v>9.416314049586775</v>
+        <v>10.36631404958678</v>
       </c>
       <c r="M38" s="4" t="n">
-        <v>24.87262809917355</v>
+        <v>25.82262809917355</v>
       </c>
       <c r="N38" s="5" t="n">
-        <v>0.2429368869936034</v>
+        <v>0.2674464818763326</v>
       </c>
       <c r="O38" s="7" t="inlineStr">
         <is>
@@ -3015,13 +3015,13 @@
         </is>
       </c>
       <c r="L39" s="4" t="n">
-        <v>9.77481818181818</v>
+        <v>10.72481818181818</v>
       </c>
       <c r="M39" s="4" t="n">
-        <v>25.58963636363636</v>
+        <v>26.53963636363636</v>
       </c>
       <c r="N39" s="5" t="n">
-        <v>0.2756999999999999</v>
+        <v>0.3024948717948718</v>
       </c>
       <c r="O39" s="7" t="inlineStr">
         <is>
@@ -3079,13 +3079,13 @@
         </is>
       </c>
       <c r="L40" s="4" t="n">
-        <v>10.89068595041322</v>
+        <v>11.84068595041323</v>
       </c>
       <c r="M40" s="4" t="n">
-        <v>27.02937190082645</v>
+        <v>28.77137190082645</v>
       </c>
       <c r="N40" s="5" t="n">
-        <v>0.2640827655310621</v>
+        <v>0.2871188376753507</v>
       </c>
       <c r="O40" s="7" t="inlineStr">
         <is>
@@ -3143,13 +3143,13 @@
         </is>
       </c>
       <c r="L41" s="4" t="n">
-        <v>9.41506611570248</v>
+        <v>11.41506611570248</v>
       </c>
       <c r="M41" s="4" t="n">
-        <v>24.87013223140496</v>
+        <v>25.82013223140496</v>
       </c>
       <c r="N41" s="5" t="n">
-        <v>0.2537244988864143</v>
+        <v>0.3076220489977728</v>
       </c>
       <c r="O41" s="7" t="inlineStr">
         <is>
@@ -3207,13 +3207,13 @@
         </is>
       </c>
       <c r="L42" s="4" t="n">
-        <v>12.48217768595041</v>
+        <v>14.48217768595041</v>
       </c>
       <c r="M42" s="4" t="n">
-        <v>31.00435537190083</v>
+        <v>31.95435537190082</v>
       </c>
       <c r="N42" s="5" t="n">
-        <v>0.2608537996545768</v>
+        <v>0.30265</v>
       </c>
       <c r="O42" s="7" t="inlineStr">
         <is>
@@ -3362,10 +3362,10 @@
         <v>37.38</v>
       </c>
       <c r="I5" s="4" t="n">
-        <v>9.970293388429759</v>
+        <v>11.97029338842976</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>0.1803296711509717</v>
+        <v>0.2165030642750375</v>
       </c>
       <c r="K5" t="n">
         <v>0.31</v>
@@ -3408,10 +3408,10 @@
         <v>34.38</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>9.73979752066116</v>
+        <v>11.73979752066116</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0.1873633545310016</v>
+        <v>0.2258371224165342</v>
       </c>
       <c r="K6" t="n">
         <v>0.23</v>
@@ -3454,10 +3454,10 @@
         <v>36.6</v>
       </c>
       <c r="I7" s="4" t="n">
-        <v>19.95278099173554</v>
+        <v>20.90278099173555</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>0.3059932192648923</v>
+        <v>0.3205622940430926</v>
       </c>
       <c r="K7" t="n">
         <v>1.05</v>
@@ -3500,10 +3500,10 @@
         <v>32.19</v>
       </c>
       <c r="I8" s="4" t="n">
-        <v>14.90079338842976</v>
+        <v>15.85079338842976</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>0.2695061285500748</v>
+        <v>0.2866884902840061</v>
       </c>
       <c r="K8" t="n">
         <v>1.24</v>
@@ -3546,10 +3546,10 @@
         <v>42.75</v>
       </c>
       <c r="I9" s="4" t="n">
-        <v>18.70902479338843</v>
+        <v>19.68102479338843</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>0.2666421672555948</v>
+        <v>0.2804951707891638</v>
       </c>
       <c r="K9" t="n">
         <v>2.02</v>
@@ -3592,10 +3592,10 @@
         <v>32.7</v>
       </c>
       <c r="I10" s="4" t="n">
-        <v>25.19802892561983</v>
+        <v>26.14802892561983</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0.3768802843016069</v>
+        <v>0.3910891841779975</v>
       </c>
       <c r="K10" t="n">
         <v>1.01</v>
@@ -3642,7 +3642,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Tramo propuesto: menos de 20 € → 5,95 €; de 20 a 39 € → 3,95 €; desde 39 € → gratis. Cubrimos así el coste real del envío del proveedor en los pedidos pequeños.</t>
+          <t>Tramo propuesto: menos de 20 € → 5,95 €; de 20 a 39 € → 3,95 €; desde 39 € → gratis. Coste real del proveedor: tarifa AW 2,95 € (≤1 kg) / 4,00 € (1-5 kg) / 6,50 € (&gt;5 kg), sin IVA.</t>
         </is>
       </c>
     </row>
@@ -3717,7 +3717,7 @@
         <v>7.073485289833965</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>4.95</v>
+        <v>2.95</v>
       </c>
       <c r="G5" s="4" t="n">
         <v>1.40275</v>
@@ -3726,10 +3726,10 @@
         <v>0.2620282148471448</v>
       </c>
       <c r="I5" s="13" t="n">
-        <v>4.575786082095751</v>
+        <v>6.575786082095751</v>
       </c>
       <c r="J5" s="5" t="n">
-        <v>0.3715906818346214</v>
+        <v>0.5340067892171717</v>
       </c>
     </row>
     <row r="6">
@@ -3751,7 +3751,7 @@
         <v>11.82079085348092</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>4.95</v>
+        <v>2.95</v>
       </c>
       <c r="G6" s="4" t="n">
         <v>1.55275</v>
@@ -3760,10 +3760,10 @@
         <v>0.4378860771606649</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>7.767085466052633</v>
+        <v>9.767085466052633</v>
       </c>
       <c r="J6" s="5" t="n">
-        <v>0.3774366832901079</v>
+        <v>0.4746254383101882</v>
       </c>
     </row>
     <row r="7">
@@ -3785,7 +3785,7 @@
         <v>15.61863530439848</v>
       </c>
       <c r="F7" s="4" t="n">
-        <v>4.95</v>
+        <v>2.95</v>
       </c>
       <c r="G7" s="4" t="n">
         <v>1.64275</v>
@@ -3794,10 +3794,10 @@
         <v>0.5785723670114807</v>
       </c>
       <c r="I7" s="13" t="n">
-        <v>8.350124973218133</v>
+        <v>10.35012497321813</v>
       </c>
       <c r="J7" s="5" t="n">
-        <v>0.3071018607171411</v>
+        <v>0.3806580917201806</v>
       </c>
     </row>
     <row r="8">
@@ -3819,7 +3819,7 @@
         <v>18.94174919895135</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>4.95</v>
+        <v>4</v>
       </c>
       <c r="G8" s="4" t="n">
         <v>1.6885</v>
@@ -3828,10 +3828,10 @@
         <v>0.701672870630945</v>
       </c>
       <c r="I8" s="13" t="n">
-        <v>6.693284541987953</v>
+        <v>7.643284541987953</v>
       </c>
       <c r="J8" s="5" t="n">
-        <v>0.2029793056592838</v>
+        <v>0.2317888294688076</v>
       </c>
     </row>
     <row r="9">
@@ -3853,7 +3853,7 @@
         <v>26.06270754442179</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>4.95</v>
+        <v>4</v>
       </c>
       <c r="G9" s="4" t="n">
         <v>1.9135</v>
@@ -3862,10 +3862,10 @@
         <v>0.9654596641012246</v>
       </c>
       <c r="I9" s="13" t="n">
-        <v>11.48023361792327</v>
+        <v>12.43023361792327</v>
       </c>
       <c r="J9" s="5" t="n">
-        <v>0.2530251853859227</v>
+        <v>0.2739632546026804</v>
       </c>
     </row>
     <row r="10">
@@ -3887,7 +3887,7 @@
         <v>33.18366588989223</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>4.95</v>
+        <v>4</v>
       </c>
       <c r="G10" s="4" t="n">
         <v>2.1385</v>
@@ -3896,10 +3896,10 @@
         <v>1.229246457571505</v>
       </c>
       <c r="I10" s="13" t="n">
-        <v>16.26718269385859</v>
+        <v>17.21718269385859</v>
       </c>
       <c r="J10" s="5" t="n">
-        <v>0.2815921467749484</v>
+        <v>0.2980370680911143</v>
       </c>
     </row>
     <row r="11">
@@ -3921,7 +3921,7 @@
         <v>42.67827701718613</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>4.95</v>
+        <v>4</v>
       </c>
       <c r="G11" s="4" t="n">
         <v>2.4385</v>
@@ -3930,10 +3930,10 @@
         <v>1.580962182198545</v>
       </c>
       <c r="I11" s="13" t="n">
-        <v>22.64978146177236</v>
+        <v>23.59978146177236</v>
       </c>
       <c r="J11" s="5" t="n">
-        <v>0.3048524534899283</v>
+        <v>0.3176388828558904</v>
       </c>
     </row>
     <row r="13">
@@ -3956,7 +3956,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Con este umbral la mayoría de pedidos llevan 2 artículos o un pack. Revisa el tramo real en tu proveedor: si te cobra más de 4,95 € por envío, sube los tramos pequeños.</t>
+          <t>Con este umbral la mayoría de pedidos llevan 2 artículos o un pack. El coste real verificado en AW Dropship España es de 2,95 € (hasta 1 kg), 4,00 € (1-5 kg) y 6,50 € (más de 5 kg), sin IVA: cobrar 5,95 € en los pedidos pequeños cubre el envío y deja margen.</t>
         </is>
       </c>
     </row>
@@ -4035,16 +4035,16 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>6.973953690240332</v>
+        <v>7.923953690240332</v>
       </c>
       <c r="C5" s="4" t="n">
-        <v>11.86641748356376</v>
+        <v>12.81641748356376</v>
       </c>
       <c r="D5" s="4" t="n">
-        <v>16.75888127688719</v>
+        <v>17.70888127688719</v>
       </c>
       <c r="E5" s="4" t="n">
-        <v>23.28216633465178</v>
+        <v>24.23216633465178</v>
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
@@ -4059,16 +4059,16 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>6.693284541987953</v>
+        <v>7.643284541987953</v>
       </c>
       <c r="C6" s="4" t="n">
-        <v>11.48023361792327</v>
+        <v>12.43023361792327</v>
       </c>
       <c r="D6" s="4" t="n">
-        <v>16.26718269385859</v>
+        <v>17.21718269385859</v>
       </c>
       <c r="E6" s="4" t="n">
-        <v>22.64978146177236</v>
+        <v>23.59978146177236</v>
       </c>
       <c r="F6" s="9" t="inlineStr">
         <is>
@@ -4083,16 +4083,16 @@
         </is>
       </c>
       <c r="B7" s="4" t="n">
-        <v>6.272280819609387</v>
+        <v>7.222280819609386</v>
       </c>
       <c r="C7" s="4" t="n">
-        <v>10.90095781946253</v>
+        <v>11.85095781946253</v>
       </c>
       <c r="D7" s="4" t="n">
-        <v>15.52963481931569</v>
+        <v>16.47963481931569</v>
       </c>
       <c r="E7" s="4" t="n">
-        <v>21.70120415245323</v>
+        <v>22.65120415245323</v>
       </c>
       <c r="F7" s="9" t="inlineStr">
         <is>
@@ -4107,16 +4107,16 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>5.991611671357009</v>
+        <v>6.941611671357008</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>10.51477395382204</v>
+        <v>11.46477395382204</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>15.03793623628709</v>
+        <v>15.98793623628709</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>21.06881927957381</v>
+        <v>22.01881927957381</v>
       </c>
       <c r="F8" s="9" t="inlineStr">
         <is>
@@ -4180,7 +4180,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>7.315587921859543</v>
+        <v>8.790587921859544</v>
       </c>
     </row>
     <row r="6">
@@ -4210,7 +4210,7 @@
         </is>
       </c>
       <c r="B8" s="16" t="n">
-        <v>29.38929889114767</v>
+        <v>24.45797731746244</v>
       </c>
     </row>
     <row r="9">
@@ -4220,7 +4220,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>1229.94215859453</v>
+        <v>1023.566350735803</v>
       </c>
     </row>
     <row r="10">
@@ -4230,7 +4230,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>882.3381882789315</v>
+        <v>1103.588188278932</v>
       </c>
     </row>
     <row r="12">

</xml_diff>